<commit_message>
Contacts sweep 03/08: +1 new, 26 updated
Incremental sweep of 26/07–03/08 (60 messages: 44 Inbox, 16 Sent, 0 Archive).

One new contact: Rishi at Keylife Financial Services. Only a single outbound
message with no deal traffic behind it, so the category is a flagged
placeholder rather than a guess.

Everyone else on this week's threads was already on the list — the Askew Road
valuation (Allsop, Knight Frank), the DNA Uxbridge extension (GB Bank,
Osborne Clarke), Elysian Stanmore, the July loan-note run (Baccata, Elite
Mobile) and two TRST enquiries REL passed on. Counts, last-seen dates and a
Baccata direct dial updated from those.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014uvaSiEgA1fu77AH9kUFoN
</commit_message>
<xml_diff>
--- a/Contact_List_REL.xlsx
+++ b/Contact_List_REL.xlsx
@@ -12,7 +12,7 @@
     <sheet name="README" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contact List'!$A$4:$L$238</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contact List'!$A$4:$L$239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L238"/>
+  <dimension ref="A1:L239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built automatically from Outlook (shyam@relfinance.co.uk) — last refreshed 2026-07-28. Refreshed weekly; do not hand-edit (see README tab).</t>
+          <t>Built automatically from Outlook (shyam@relfinance.co.uk) — last refreshed 2026-08-03. Refreshed weekly; do not hand-edit (see README tab).</t>
         </is>
       </c>
     </row>
@@ -3630,11 +3630,11 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I61" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J61" s="6" t="n">
         <v>0</v>
@@ -3984,11 +3984,11 @@
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I68" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J68" s="6" t="n">
         <v>0</v>
@@ -4038,11 +4038,11 @@
       </c>
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I69" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J69" s="6" t="n">
         <v>0</v>
@@ -4678,11 +4678,11 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I81" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J81" s="6" t="n">
         <v>0</v>
@@ -4824,7 +4824,7 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I84" s="6" t="n">
@@ -4916,7 +4916,7 @@
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I86" s="6" t="n">
@@ -7934,7 +7934,7 @@
         </is>
       </c>
       <c r="I143" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J143" s="6" t="n">
         <v>0</v>
@@ -9266,14 +9266,14 @@
       </c>
       <c r="H169" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I169" s="6" t="n">
         <v>5</v>
       </c>
       <c r="J169" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K169" s="4" t="inlineStr">
         <is>
@@ -9414,7 +9414,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>+44 (0) 1534 870670</t>
+          <t>+44 (0) 1534 870670, +44 (0) 1534 870600</t>
         </is>
       </c>
       <c r="G172" s="6" t="inlineStr">
@@ -9424,14 +9424,14 @@
       </c>
       <c r="H172" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I172" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J172" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K172" s="4" t="inlineStr">
         <is>
@@ -9482,14 +9482,14 @@
       </c>
       <c r="H173" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I173" s="6" t="n">
         <v>12</v>
       </c>
       <c r="J173" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K173" s="4" t="inlineStr">
         <is>
@@ -9594,14 +9594,14 @@
       </c>
       <c r="H175" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I175" s="6" t="n">
         <v>2</v>
       </c>
       <c r="J175" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K175" s="4" t="inlineStr">
         <is>
@@ -9644,14 +9644,14 @@
       </c>
       <c r="H176" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I176" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J176" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K176" s="4" t="inlineStr">
         <is>
@@ -9694,14 +9694,14 @@
       </c>
       <c r="H177" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I177" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J177" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K177" s="4" t="inlineStr">
         <is>
@@ -9744,14 +9744,14 @@
       </c>
       <c r="H178" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I178" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J178" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K178" s="4" t="inlineStr">
         <is>
@@ -9794,14 +9794,14 @@
       </c>
       <c r="H179" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I179" s="6" t="n">
         <v>1</v>
       </c>
       <c r="J179" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K179" s="4" t="inlineStr">
         <is>
@@ -10040,14 +10040,14 @@
       </c>
       <c r="H184" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I184" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J184" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K184" s="4" t="inlineStr">
         <is>
@@ -10086,14 +10086,14 @@
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I185" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J185" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K185" s="4" t="inlineStr">
         <is>
@@ -10132,14 +10132,14 @@
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I186" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J186" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K186" s="4" t="inlineStr">
         <is>
@@ -10498,11 +10498,11 @@
       </c>
       <c r="H193" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I193" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J193" s="6" t="n">
         <v>0</v>
@@ -10822,11 +10822,11 @@
       </c>
       <c r="H199" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I199" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J199" s="6" t="n">
         <v>0</v>
@@ -10872,7 +10872,7 @@
       </c>
       <c r="H200" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I200" s="6" t="n">
@@ -11716,14 +11716,14 @@
       </c>
       <c r="H216" s="6" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I216" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J216" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K216" s="4" t="inlineStr">
         <is>
@@ -12198,14 +12198,14 @@
       </c>
       <c r="H225" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I225" s="6" t="n">
-        <v>476</v>
+        <v>492</v>
       </c>
       <c r="J225" s="6" t="n">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="K225" s="4" t="inlineStr">
         <is>
@@ -12256,14 +12256,14 @@
       </c>
       <c r="H226" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I226" s="6" t="n">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="J226" s="6" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="K226" s="4" t="inlineStr">
         <is>
@@ -12329,7 +12329,7 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>Abdul Rashid</t>
+          <t>Rishi</t>
         </is>
       </c>
       <c r="B228" s="17" t="inlineStr">
@@ -12337,29 +12337,33 @@
           <t>Personal / Other</t>
         </is>
       </c>
-      <c r="C228" s="4" t="inlineStr"/>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>Keylife Financial Services</t>
+        </is>
+      </c>
       <c r="D228" s="4" t="inlineStr"/>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>qabdul1rash1@gmail.com</t>
+          <t>rishi@keylifefs.com</t>
         </is>
       </c>
       <c r="F228" s="4" t="inlineStr"/>
       <c r="G228" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="H228" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I228" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J228" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K228" s="4" t="inlineStr">
         <is>
@@ -12368,14 +12372,14 @@
       </c>
       <c r="L228" s="8" t="inlineStr">
         <is>
-          <t>Recipient of Shyam's personal "bag radar log" file share</t>
+          <t>New contact 30/07 — Shyam sent his work email and the REL website. No deal traffic yet, so the category is a placeholder; correct it once his role is clear.</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>Anish Vora</t>
+          <t>Abdul Rashid</t>
         </is>
       </c>
       <c r="B229" s="17" t="inlineStr">
@@ -12387,37 +12391,41 @@
       <c r="D229" s="4" t="inlineStr"/>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>anishvora18@gmail.com</t>
+          <t>qabdul1rash1@gmail.com</t>
         </is>
       </c>
       <c r="F229" s="4" t="inlineStr"/>
       <c r="G229" s="6" t="inlineStr">
         <is>
-          <t>2025-06-24</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="H229" s="6" t="inlineStr">
         <is>
-          <t>2025-06-24</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="I229" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J229" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K229" s="7" t="inlineStr">
-        <is>
-          <t>Named in a thread</t>
-        </is>
-      </c>
-      <c r="L229" s="8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K229" s="4" t="inlineStr">
+        <is>
+          <t>Direct correspondence</t>
+        </is>
+      </c>
+      <c r="L229" s="8" t="inlineStr">
+        <is>
+          <t>Recipient of Shyam's personal "bag radar log" file share</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>Chloe</t>
+          <t>Anish Vora</t>
         </is>
       </c>
       <c r="B230" s="17" t="inlineStr">
@@ -12429,18 +12437,18 @@
       <c r="D230" s="4" t="inlineStr"/>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>chloej0027@gmail.com</t>
+          <t>anishvora18@gmail.com</t>
         </is>
       </c>
       <c r="F230" s="4" t="inlineStr"/>
       <c r="G230" s="6" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2025-06-24</t>
         </is>
       </c>
       <c r="H230" s="6" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2025-06-24</t>
         </is>
       </c>
       <c r="I230" s="6" t="n">
@@ -12459,7 +12467,7 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>Darren Halcrow</t>
+          <t>Chloe</t>
         </is>
       </c>
       <c r="B231" s="17" t="inlineStr">
@@ -12471,41 +12479,37 @@
       <c r="D231" s="4" t="inlineStr"/>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>darren.halcrow@hotmail.co.uk</t>
+          <t>chloej0027@gmail.com</t>
         </is>
       </c>
       <c r="F231" s="4" t="inlineStr"/>
       <c r="G231" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="H231" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="I231" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J231" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K231" s="4" t="inlineStr">
-        <is>
-          <t>Direct correspondence</t>
-        </is>
-      </c>
-      <c r="L231" s="8" t="inlineStr">
-        <is>
-          <t>Recipient of Shyam's personal "bag radar log" file share</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K231" s="7" t="inlineStr">
+        <is>
+          <t>Named in a thread</t>
+        </is>
+      </c>
+      <c r="L231" s="8" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>Deepesh Thakrar</t>
+          <t>Darren Halcrow</t>
         </is>
       </c>
       <c r="B232" s="17" t="inlineStr">
@@ -12517,37 +12521,41 @@
       <c r="D232" s="4" t="inlineStr"/>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>dc.thakrar@gmail.com</t>
+          <t>darren.halcrow@hotmail.co.uk</t>
         </is>
       </c>
       <c r="F232" s="4" t="inlineStr"/>
       <c r="G232" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="H232" s="6" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="I232" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J232" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K232" s="7" t="inlineStr">
-        <is>
-          <t>Named in a thread</t>
-        </is>
-      </c>
-      <c r="L232" s="8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K232" s="4" t="inlineStr">
+        <is>
+          <t>Direct correspondence</t>
+        </is>
+      </c>
+      <c r="L232" s="8" t="inlineStr">
+        <is>
+          <t>Recipient of Shyam's personal "bag radar log" file share</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>Gary Brooks</t>
+          <t>Deepesh Thakrar</t>
         </is>
       </c>
       <c r="B233" s="17" t="inlineStr">
@@ -12559,41 +12567,37 @@
       <c r="D233" s="4" t="inlineStr"/>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>garyjbrooks@gmail.com</t>
+          <t>dc.thakrar@gmail.com</t>
         </is>
       </c>
       <c r="F233" s="4" t="inlineStr"/>
       <c r="G233" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H233" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="I233" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J233" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K233" s="4" t="inlineStr">
-        <is>
-          <t>Direct correspondence</t>
-        </is>
-      </c>
-      <c r="L233" s="8" t="inlineStr">
-        <is>
-          <t>Recipient of Shyam's personal "bag radar log" file share</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K233" s="7" t="inlineStr">
+        <is>
+          <t>Named in a thread</t>
+        </is>
+      </c>
+      <c r="L233" s="8" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>J Crypto</t>
+          <t>Gary Brooks</t>
         </is>
       </c>
       <c r="B234" s="17" t="inlineStr">
@@ -12605,37 +12609,41 @@
       <c r="D234" s="4" t="inlineStr"/>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>jcrypto401@gmail.com</t>
+          <t>garyjbrooks@gmail.com</t>
         </is>
       </c>
       <c r="F234" s="4" t="inlineStr"/>
       <c r="G234" s="6" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="H234" s="6" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="I234" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J234" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K234" s="4" t="inlineStr">
         <is>
           <t>Direct correspondence</t>
         </is>
       </c>
-      <c r="L234" s="8" t="inlineStr"/>
+      <c r="L234" s="8" t="inlineStr">
+        <is>
+          <t>Recipient of Shyam's personal "bag radar log" file share</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>Joel Smart</t>
+          <t>J Crypto</t>
         </is>
       </c>
       <c r="B235" s="17" t="inlineStr">
@@ -12647,41 +12655,37 @@
       <c r="D235" s="4" t="inlineStr"/>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>joelsmart2023@gmail.com</t>
+          <t>jcrypto401@gmail.com</t>
         </is>
       </c>
       <c r="F235" s="4" t="inlineStr"/>
       <c r="G235" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="H235" s="6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="I235" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J235" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K235" s="4" t="inlineStr">
         <is>
           <t>Direct correspondence</t>
         </is>
       </c>
-      <c r="L235" s="8" t="inlineStr">
-        <is>
-          <t>Recipient of Shyam's personal "bag radar log" file share</t>
-        </is>
-      </c>
+      <c r="L235" s="8" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>Malus Entity</t>
+          <t>Joel Smart</t>
         </is>
       </c>
       <c r="B236" s="17" t="inlineStr">
@@ -12693,7 +12697,7 @@
       <c r="D236" s="4" t="inlineStr"/>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>malus.entity@gmail.com</t>
+          <t>joelsmart2023@gmail.com</t>
         </is>
       </c>
       <c r="F236" s="4" t="inlineStr"/>
@@ -12727,7 +12731,7 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>Shyam Lakhani</t>
+          <t>Malus Entity</t>
         </is>
       </c>
       <c r="B237" s="17" t="inlineStr">
@@ -12739,25 +12743,25 @@
       <c r="D237" s="4" t="inlineStr"/>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>slakhani0203@gmail.com</t>
+          <t>malus.entity@gmail.com</t>
         </is>
       </c>
       <c r="F237" s="4" t="inlineStr"/>
       <c r="G237" s="6" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="H237" s="6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="I237" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J237" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K237" s="4" t="inlineStr">
         <is>
@@ -12766,7 +12770,7 @@
       </c>
       <c r="L237" s="8" t="inlineStr">
         <is>
-          <t>Mailbox owner's personal Gmail; REL Finance employment offer correspondence.</t>
+          <t>Recipient of Shyam's personal "bag radar log" file share</t>
         </is>
       </c>
     </row>
@@ -12785,25 +12789,25 @@
       <c r="D238" s="4" t="inlineStr"/>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>shyam_302@hotmail.co.uk</t>
+          <t>slakhani0203@gmail.com</t>
         </is>
       </c>
       <c r="F238" s="4" t="inlineStr"/>
       <c r="G238" s="6" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="H238" s="6" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I238" s="6" t="n">
         <v>3</v>
       </c>
       <c r="J238" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K238" s="4" t="inlineStr">
         <is>
@@ -12812,12 +12816,58 @@
       </c>
       <c r="L238" s="8" t="inlineStr">
         <is>
+          <t>Mailbox owner's personal Gmail; REL Finance employment offer correspondence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>Shyam Lakhani</t>
+        </is>
+      </c>
+      <c r="B239" s="17" t="inlineStr">
+        <is>
+          <t>Personal / Other</t>
+        </is>
+      </c>
+      <c r="C239" s="4" t="inlineStr"/>
+      <c r="D239" s="4" t="inlineStr"/>
+      <c r="E239" s="4" t="inlineStr">
+        <is>
+          <t>shyam_302@hotmail.co.uk</t>
+        </is>
+      </c>
+      <c r="F239" s="4" t="inlineStr"/>
+      <c r="G239" s="6" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="H239" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I239" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J239" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K239" s="4" t="inlineStr">
+        <is>
+          <t>Direct correspondence</t>
+        </is>
+      </c>
+      <c r="L239" s="8" t="inlineStr">
+        <is>
           <t>Mailbox owner's own personal Hotmail address</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L238"/>
+  <autoFilter ref="A4:L239"/>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
@@ -12865,7 +12915,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A4)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A4)</f>
         <v/>
       </c>
     </row>
@@ -12876,7 +12926,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A5)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A5)</f>
         <v/>
       </c>
     </row>
@@ -12887,7 +12937,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A6)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A6)</f>
         <v/>
       </c>
     </row>
@@ -12898,7 +12948,7 @@
         </is>
       </c>
       <c r="B7" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A7)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A7)</f>
         <v/>
       </c>
     </row>
@@ -12909,7 +12959,7 @@
         </is>
       </c>
       <c r="B8" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A8)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A8)</f>
         <v/>
       </c>
     </row>
@@ -12920,7 +12970,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A9)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A9)</f>
         <v/>
       </c>
     </row>
@@ -12931,7 +12981,7 @@
         </is>
       </c>
       <c r="B10" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A10)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A10)</f>
         <v/>
       </c>
     </row>
@@ -12942,7 +12992,7 @@
         </is>
       </c>
       <c r="B11" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A11)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A11)</f>
         <v/>
       </c>
     </row>
@@ -12953,7 +13003,7 @@
         </is>
       </c>
       <c r="B12" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A12)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A12)</f>
         <v/>
       </c>
     </row>
@@ -12964,7 +13014,7 @@
         </is>
       </c>
       <c r="B13" s="21">
-        <f>COUNTIF('Contact List'!$B$5:$B$238,A13)</f>
+        <f>COUNTIF('Contact List'!$B$5:$B$239,A13)</f>
         <v/>
       </c>
     </row>

</xml_diff>